<commit_message>
Add the Payoff tab
Scenario payoffs for both expressions with an expected value, sizing against
the rates sleeve, and a falsification calendar that puts a date and a number
on every way the trade can be wrong.

The conditional structure pays only where the 2-year is what rallies, so its
payoff column returns premium-only whenever the curve steepens from the long
end. That is the whole reason for preferring it, and the sheet now shows it
rather than asserting it.

The July minutes have several Board members expecting inflation to
accelerate in the second half of the fiscal year. That is the strongest
argument against the trade, it is testable on known dates, and it is on the
calendar with the print that would end the position.
</commit_message>
<xml_diff>
--- a/JPY_Bull_Steepener.xlsx
+++ b/JPY_Bull_Steepener.xlsx
@@ -14,7 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CurveSlope" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BullSteepener" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JPYEvidence" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MacroLink" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payoff" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MacroLink" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="AsOf">Control!$B$6</definedName>
@@ -33,7 +34,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="dd-mmm-yyyy"/>
     <numFmt numFmtId="165" formatCode="+0.00;-0.00"/>
     <numFmt numFmtId="166" formatCode="+#,##0;-#,##0"/>
@@ -42,8 +43,9 @@
     <numFmt numFmtId="169" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="170" formatCode="dd-mmm-yy"/>
     <numFmt numFmtId="171" formatCode="0.0"/>
+    <numFmt numFmtId="172" formatCode="+#,##0.0;-#,##0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,6 +92,11 @@
       <color rgb="00DB0011"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00DB0011"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -126,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -178,6 +185,15 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -1178,6 +1194,425 @@
                 </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:rPr>
+              <a:t>Payoff by state, bp of 2s10s</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>Cash 2s10s spread</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="DB0011"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Payoff'!$A$21:$A$25</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Payoff'!$F$21:$F$25</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>6m conditional steepener</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="44546A"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Payoff'!$A$21:$A$25</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Payoff'!$G$21:$G$25</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <numFmt formatCode="+#,##0;-#,##0"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="1000" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Arial"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t/>
+              </a:r>
+              <a:endParaRPr sz="1000" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:endParaRPr>
+            </a:p>
+          </txPr>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="60"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D0CECE"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="950" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="767576"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="767576"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D0CECE"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="950" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="767576"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="767576"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+      <overlay val="0"/>
+      <txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:t/>
+          </a:r>
+          <a:endParaRPr sz="950" b="0">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:latin typeface="Arial"/>
+          </a:endParaRPr>
+        </a:p>
+      </txPr>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+  <spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:noFill/>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>Probability by state</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="44546A"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Payoff'!$A$21:$A$25</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Payoff'!$B$21:$B$25</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <numFmt formatCode="0%"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="1000" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Arial"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t/>
+              </a:r>
+              <a:endParaRPr sz="1000" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:endParaRPr>
+            </a:p>
+          </txPr>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="60"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D0CECE"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="950" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="767576"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="767576"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D0CECE"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="950" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="767576"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="767576"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+  <spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:noFill/>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:rPr>
               <a:t>Headline against core — US and Japan, % y/y</a:t>
             </a:r>
           </a:p>
@@ -1337,7 +1772,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -1519,7 +1954,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart17.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -4273,6 +4708,55 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>7</col>
       <colOff>0</colOff>
       <row>4</row>
@@ -4629,7 +5113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4740,59 +5224,71 @@
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
+          <t>Payoff</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>What it makes by state of the world, an expected value for both expressions, sizing against the rates sleeve, and a falsification calendar with a date and a number on every line. Two charts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
           <t>MacroLink</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>The artefacts that tie the trade to the macro framing: channel-to-instrument map, scenario strip, positioning table, and three charts. Three charts, three tables.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>How to run it</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>1.  Open on the Bloomberg laptop and confirm the ribbon is present.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>2.  Control tab — set the as-of date, or leave =TODAY() for a live book.</t>
+          <t>1.  Open on the Bloomberg laptop and confirm the ribbon is present.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>3.  Bloomberg &gt; Refresh &gt; Refresh Entire Workbook.</t>
+          <t>2.  Control tab — set the as-of date, or leave =TODAY() for a live book.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>4.  Check the date alignment cell near the top of each tab reads 0 / OK before trusting a number.</t>
+          <t>3.  Bloomberg &gt; Refresh &gt; Refresh Entire Workbook.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="7" t="inlineStr">
         <is>
+          <t>4.  Check the date alignment cell near the top of each tab reads 0 / OK before trusting a number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
           <t>5.  The charts redraw themselves — they point at the ranges the formulas spill into, not at pasted values.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>This file is a build artefact. It is generated by data-puller/build_data_puller.py alongside the full Q2 book and shares every sheet builder with it, so the two cannot disagree. Never repair it by hand — fix the script and rebuild, or the fix is lost the next time anyone regenerates it.</t>
         </is>
@@ -33871,6 +34367,854 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Payoff, sizing, and the dates that settle it</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Scenario payoffs for both expressions, an expected value, and a falsification calendar with the number that ends the trade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="4" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Inputs — shaded cells are yours to set on the terminal</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Entry level, 2s10s bp</t>
+        </is>
+      </c>
+      <c r="B6" s="17">
+        <f>IFERROR(BullSteepener!C18,"")</f>
+        <v/>
+      </c>
+      <c r="H6" s="32" t="inlineStr">
+        <is>
+          <t>Defaults to spot. Overwrite with your fill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Target, bp</t>
+        </is>
+      </c>
+      <c r="B7" s="17">
+        <f>IFERROR(BullSteepener!B49,"")</f>
+        <v/>
+      </c>
+      <c r="H7" s="32" t="inlineStr">
+        <is>
+          <t>From the mean-reversion block on BullSteepener.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Stop, bp</t>
+        </is>
+      </c>
+      <c r="B8" s="17">
+        <f>IFERROR(BullSteepener!B51,"")</f>
+        <v/>
+      </c>
+      <c r="H8" s="32" t="inlineStr">
+        <is>
+          <t>As above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Carry and roll, bp per quarter</t>
+        </is>
+      </c>
+      <c r="B9" s="17">
+        <f>IFERROR(BullSteepener!C84,"")</f>
+        <v/>
+      </c>
+      <c r="H9" s="32" t="inlineStr">
+        <is>
+          <t>Computed off the live curve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Horizon, quarters</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="32" t="inlineStr">
+        <is>
+          <t>Two quarters spans the Sep and Oct meetings and three core-core prints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Conditional premium, bp</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="H11" s="32" t="inlineStr">
+        <is>
+          <t>6m conditional bull steepener, receiver spread. JPY swaptions are quoted in NORMAL (Bachelier) vol in basis points, so price it off the vol surface and put the premium here in bp of notional. 18 is a placeholder until you do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Conditional strike, bp of steepening</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="H12" s="32" t="inlineStr">
+        <is>
+          <t>How far the curve must steepen before the structure pays.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Book size, $m</t>
+        </is>
+      </c>
+      <c r="B13" s="41" t="n">
+        <v>100</v>
+      </c>
+      <c r="H13" s="32" t="inlineStr">
+        <is>
+          <t>For the sizing block below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Rates sleeve, % of book</t>
+        </is>
+      </c>
+      <c r="B14" s="42" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H14" s="32" t="inlineStr">
+        <is>
+          <t>Trade 2 carries 30% in the macro deck. This shares that sleeve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>What it makes, by state of the world</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Probabilities are the author's, over the BoJ path rather than over the macro scenarios in the main deck — they are a different partition and should not be confused with the 55 / 25 / 20. The 2y and 10y moves are the assumption; everything to the right of them is arithmetic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Prob.</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>2y move, bp</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>10y move, bp</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>2s10s outcome</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Cash P&amp;L, bp</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Conditional P&amp;L, bp</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>BoJ pauses — bull steepening</t>
+        </is>
+      </c>
+      <c r="B21" s="43" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C21" s="35" t="n">
+        <v>-45</v>
+      </c>
+      <c r="D21" s="35" t="n">
+        <v>-3</v>
+      </c>
+      <c r="E21" s="35">
+        <f>IFERROR($B$6+(D21-C21),"")</f>
+        <v/>
+      </c>
+      <c r="F21" s="25">
+        <f>IFERROR((E21-$B$6)+$B$9*$B$10,"")</f>
+        <v/>
+      </c>
+      <c r="G21" s="25">
+        <f>IFERROR(IF(C21&lt;0,MAX(0,(E21-$B$6)-$B$12),0)-$B$11,"")</f>
+        <v/>
+      </c>
+      <c r="H21" s="32" t="inlineStr">
+        <is>
+          <t>The front end hands back the priced hikes. The state the trade is underwriting, and the only one where the conditional pays.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Nothing happens — carry</t>
+        </is>
+      </c>
+      <c r="B22" s="43" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C22" s="35" t="n">
+        <v>-5</v>
+      </c>
+      <c r="D22" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="35">
+        <f>IFERROR($B$6+(D22-C22),"")</f>
+        <v/>
+      </c>
+      <c r="F22" s="25">
+        <f>IFERROR((E22-$B$6)+$B$9*$B$10,"")</f>
+        <v/>
+      </c>
+      <c r="G22" s="25">
+        <f>IFERROR(IF(C22&lt;0,MAX(0,(E22-$B$6)-$B$12),0)-$B$11,"")</f>
+        <v/>
+      </c>
+      <c r="H22" s="32" t="inlineStr">
+        <is>
+          <t>The curve drifts. You collect carry and roll, and the conditional expires worthless.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Supply-led bear steepening</t>
+        </is>
+      </c>
+      <c r="B23" s="43" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C23" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="D23" s="35" t="n">
+        <v>37</v>
+      </c>
+      <c r="E23" s="35">
+        <f>IFERROR($B$6+(D23-C23),"")</f>
+        <v/>
+      </c>
+      <c r="F23" s="25">
+        <f>IFERROR((E23-$B$6)+$B$9*$B$10,"")</f>
+        <v/>
+      </c>
+      <c r="G23" s="25">
+        <f>IFERROR(IF(C23&lt;0,MAX(0,(E23-$B$6)-$B$12),0)-$B$11,"")</f>
+        <v/>
+      </c>
+      <c r="H23" s="32" t="inlineStr">
+        <is>
+          <t>The consensus JGB trade. The cash spread is along for the ride; the conditional is not, because the front end never rallies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>BoJ delivers — bear flattening</t>
+        </is>
+      </c>
+      <c r="B24" s="43" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C24" s="35" t="n">
+        <v>30</v>
+      </c>
+      <c r="D24" s="35" t="n">
+        <v>7</v>
+      </c>
+      <c r="E24" s="35">
+        <f>IFERROR($B$6+(D24-C24),"")</f>
+        <v/>
+      </c>
+      <c r="F24" s="25">
+        <f>IFERROR((E24-$B$6)+$B$9*$B$10,"")</f>
+        <v/>
+      </c>
+      <c r="G24" s="25">
+        <f>IFERROR(IF(C24&lt;0,MAX(0,(E24-$B$6)-$B$12),0)-$B$11,"")</f>
+        <v/>
+      </c>
+      <c r="H24" s="32" t="inlineStr">
+        <is>
+          <t>Sep and Oct hikes land. The cash spread loses; the conditional loses premium only. This is the state the July minutes point to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Risk-off bull flattening</t>
+        </is>
+      </c>
+      <c r="B25" s="43" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C25" s="35" t="n">
+        <v>-10</v>
+      </c>
+      <c r="D25" s="35" t="n">
+        <v>-28</v>
+      </c>
+      <c r="E25" s="35">
+        <f>IFERROR($B$6+(D25-C25),"")</f>
+        <v/>
+      </c>
+      <c r="F25" s="25">
+        <f>IFERROR((E25-$B$6)+$B$9*$B$10,"")</f>
+        <v/>
+      </c>
+      <c r="G25" s="25">
+        <f>IFERROR(IF(C25&lt;0,MAX(0,(E25-$B$6)-$B$12),0)-$B$11,"")</f>
+        <v/>
+      </c>
+      <c r="H25" s="32" t="inlineStr">
+        <is>
+          <t>A global duration rally where the long end leads. The one state where both legs of the cash spread work against you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Expected value</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>Probability check</t>
+        </is>
+      </c>
+      <c r="B28" s="27">
+        <f>SUM($B$21:$B$25)</f>
+        <v/>
+      </c>
+      <c r="H28" s="32" t="inlineStr">
+        <is>
+          <t>Must be 100%. If it is not, the numbers below mean nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Cash spread, expected bp</t>
+        </is>
+      </c>
+      <c r="B29" s="44">
+        <f>SUMPRODUCT($B$21:$B$25,$F$21:$F$25)</f>
+        <v/>
+      </c>
+      <c r="H29" s="32" t="inlineStr">
+        <is>
+          <t>Probability-weighted, including carry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Conditional, expected bp</t>
+        </is>
+      </c>
+      <c r="B30" s="44">
+        <f>SUMPRODUCT($B$21:$B$25,$G$21:$G$25)</f>
+        <v/>
+      </c>
+      <c r="H30" s="32" t="inlineStr">
+        <is>
+          <t>Probability-weighted, net of premium.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>Cash — probability of loss</t>
+        </is>
+      </c>
+      <c r="B31" s="27">
+        <f>SUMIF($F$21:$F$25,"&lt;0",$B$21:$B$25)</f>
+        <v/>
+      </c>
+      <c r="H31" s="32" t="inlineStr">
+        <is>
+          <t>How often the cash spread is a losing trade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>Conditional — probability of loss</t>
+        </is>
+      </c>
+      <c r="B32" s="27">
+        <f>SUMIF($G$21:$G$25,"&lt;0",$B$21:$B$25)</f>
+        <v/>
+      </c>
+      <c r="H32" s="32" t="inlineStr">
+        <is>
+          <t>Higher hit rate of small losses, and that is the point — the losses are capped at premium.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>Cash — worst state, bp</t>
+        </is>
+      </c>
+      <c r="B33" s="25">
+        <f>MIN($F$21:$F$25)</f>
+        <v/>
+      </c>
+      <c r="H33" s="32" t="inlineStr">
+        <is>
+          <t>Compare with the stop. If the worst state is beyond the stop, the stop is what you actually own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>Conditional — worst state, bp</t>
+        </is>
+      </c>
+      <c r="B34" s="25">
+        <f>MIN($G$21:$G$25)</f>
+        <v/>
+      </c>
+      <c r="H34" s="32" t="inlineStr">
+        <is>
+          <t>Premium, by construction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="44" customHeight="1">
+      <c r="A36" s="24">
+        <f>IF(COUNT($F$21:$G$25)=0,"Set the inputs and this reads itself.","Expected value: "&amp;TEXT(SUMPRODUCT($B$21:$B$25,$F$21:$F$25),"+0.0;-0.0")&amp;"bp on the cash spread against "&amp;TEXT(SUMPRODUCT($B$21:$B$25,$G$21:$G$25),"+0.0;-0.0")&amp;"bp on the conditional — but the cash spread loses in "&amp;TEXT(SUMIF($F$21:$F$25,"&lt;0",$B$21:$B$25),"0%")&amp;" of states against "&amp;TEXT(SUMIF($G$21:$G$25,"&lt;0",$B$21:$B$25),"0%")&amp;" for the conditional, and its worst state is "&amp;TEXT(MIN($F$21:$F$25),"0")&amp;"bp against a capped "&amp;TEXT(MIN($G$21:$G$25),"0")&amp;"bp.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Sizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>Rates sleeve, $m</t>
+        </is>
+      </c>
+      <c r="B40" s="31">
+        <f>IFERROR($B$13*$B$14,"")</f>
+        <v/>
+      </c>
+      <c r="H40" s="32" t="inlineStr">
+        <is>
+          <t>The sleeve this trade shares with the US 5s30s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>Distance to stop, bp</t>
+        </is>
+      </c>
+      <c r="B41" s="34">
+        <f>IFERROR($B$6-$B$8,"")</f>
+        <v/>
+      </c>
+      <c r="H41" s="32" t="inlineStr">
+        <is>
+          <t>Entry less stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>Cash — max loss at stop, $m</t>
+        </is>
+      </c>
+      <c r="B42" s="45">
+        <f>IFERROR($B$40*ABS($B$41)/10000*10,"")</f>
+        <v/>
+      </c>
+      <c r="H42" s="32" t="inlineStr">
+        <is>
+          <t>At a DV01 sized so a 10bp adverse move costs 0.1% of the sleeve. Replace the factor with your desk's DV01 convention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>Cash — max loss, % of book</t>
+        </is>
+      </c>
+      <c r="B43" s="46">
+        <f>IFERROR($B$42/$B$13,"")</f>
+        <v/>
+      </c>
+      <c r="H43" s="32" t="inlineStr">
+        <is>
+          <t>The number the PM actually asks for.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>Conditional — max loss, $m</t>
+        </is>
+      </c>
+      <c r="B44" s="45">
+        <f>IFERROR($B$40*$B$11/10000*10,"")</f>
+        <v/>
+      </c>
+      <c r="H44" s="32" t="inlineStr">
+        <is>
+          <t>Premium only, and it is known on day one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="inlineStr">
+        <is>
+          <t>Conditional — max loss, % of book</t>
+        </is>
+      </c>
+      <c r="B45" s="46">
+        <f>IFERROR($B$44/$B$13,"")</f>
+        <v/>
+      </c>
+      <c r="H45" s="32" t="inlineStr">
+        <is>
+          <t>Pre-sized, no stop required, survives a gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>The falsification calendar — dated, with the number</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>The July minutes show several Board members expecting inflation to accelerate significantly in the second half of the fiscal year, and two favouring faster hikes on firms' willingness to raise prices. That is the strongest argument against this trade and it is testable on a known date. Our reading is that broad-based price increases are cost pass-through from the same crude shock the April Outlook says will wane — so core-core is the arbiter, not headline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>What kills the trade</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr"/>
+      <c r="E51" s="9" t="inlineStr"/>
+      <c r="F51" s="9" t="inlineStr"/>
+      <c r="G51" s="9" t="inlineStr"/>
+      <c r="H51" s="9" t="inlineStr">
+        <is>
+          <t>What confirms it</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>18 Sep 2026</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>BoJ policy meeting</t>
+        </is>
+      </c>
+      <c r="C52" s="47" t="inlineStr">
+        <is>
+          <t>A hike delivered WITH hawkish guidance on the path</t>
+        </is>
+      </c>
+      <c r="D52" s="19" t="n"/>
+      <c r="E52" s="19" t="n"/>
+      <c r="F52" s="19" t="n"/>
+      <c r="G52" s="19" t="n"/>
+      <c r="H52" s="32" t="inlineStr">
+        <is>
+          <t>A hike delivered as a one-and-done — that is the entry, not the exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>Sep / Oct / Nov</t>
+        </is>
+      </c>
+      <c r="B53" s="17" t="inlineStr">
+        <is>
+          <t>National core-core CPI, monthly</t>
+        </is>
+      </c>
+      <c r="C53" s="47" t="inlineStr">
+        <is>
+          <t>Two consecutive prints back above 2.2% and rising</t>
+        </is>
+      </c>
+      <c r="D53" s="19" t="n"/>
+      <c r="E53" s="19" t="n"/>
+      <c r="F53" s="19" t="n"/>
+      <c r="G53" s="19" t="n"/>
+      <c r="H53" s="32" t="inlineStr">
+        <is>
+          <t>Core-core holding at or below 2% while headline stays crude-driven</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B54" s="17" t="inlineStr">
+        <is>
+          <t>BoJ policy meeting and Outlook Report</t>
+        </is>
+      </c>
+      <c r="C54" s="47" t="inlineStr">
+        <is>
+          <t>The FY27 CPI forecast revised UP</t>
+        </is>
+      </c>
+      <c r="D54" s="19" t="n"/>
+      <c r="E54" s="19" t="n"/>
+      <c r="F54" s="19" t="n"/>
+      <c r="G54" s="19" t="n"/>
+      <c r="H54" s="32" t="inlineStr">
+        <is>
+          <t>The FY27 forecast held or cut, confirming the terms-of-trade read</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="B55" s="17" t="inlineStr">
+        <is>
+          <t>USD/JPY against 165</t>
+        </is>
+      </c>
+      <c r="C55" s="47" t="inlineStr">
+        <is>
+          <t>Through 165 and holding — the BoJ hikes for FX regardless of growth</t>
+        </is>
+      </c>
+      <c r="D55" s="19" t="n"/>
+      <c r="E55" s="19" t="n"/>
+      <c r="F55" s="19" t="n"/>
+      <c r="G55" s="19" t="n"/>
+      <c r="H55" s="32" t="inlineStr">
+        <is>
+          <t>Held below 160 after the coordinated intervention</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="B56" s="17" t="inlineStr">
+        <is>
+          <t>Real wages and household spending</t>
+        </is>
+      </c>
+      <c r="C56" s="47" t="inlineStr">
+        <is>
+          <t>Spending turns positive while real wages keep rising</t>
+        </is>
+      </c>
+      <c r="D56" s="19" t="n"/>
+      <c r="E56" s="19" t="n"/>
+      <c r="F56" s="19" t="n"/>
+      <c r="G56" s="19" t="n"/>
+      <c r="H56" s="32" t="inlineStr">
+        <is>
+          <t>The divergence persists — income rising, spending falling</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>Spring 2027</t>
+        </is>
+      </c>
+      <c r="B57" s="17" t="inlineStr">
+        <is>
+          <t>Shunto first tally</t>
+        </is>
+      </c>
+      <c r="C57" s="47" t="inlineStr">
+        <is>
+          <t>Above 5.5% again, making the wage impulse durable</t>
+        </is>
+      </c>
+      <c r="D57" s="19" t="n"/>
+      <c r="E57" s="19" t="n"/>
+      <c r="F57" s="19" t="n"/>
+      <c r="G57" s="19" t="n"/>
+      <c r="H57" s="32" t="inlineStr">
+        <is>
+          <t>Below 5%, and the wage-price loop is not self-sustaining</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>Every line has a date and a number. A thesis without either is a view, and a view is not a trade — it is the thing you defend after it has gone wrong.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -33943,27 +35287,27 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="41" t="inlineStr">
+      <c r="A7" s="48" t="inlineStr">
         <is>
           <t>1 · Fed / discount rate</t>
         </is>
       </c>
-      <c r="B7" s="42" t="inlineStr">
+      <c r="B7" s="49" t="inlineStr">
         <is>
           <t>UST 10y 3.97 → 4.71%</t>
         </is>
       </c>
-      <c r="C7" s="42" t="inlineStr">
+      <c r="C7" s="49" t="inlineStr">
         <is>
           <t>US 5s30s steepener</t>
         </is>
       </c>
-      <c r="D7" s="42" t="inlineStr">
+      <c r="D7" s="49" t="inlineStr">
         <is>
           <t>Bear steepener</t>
         </is>
       </c>
-      <c r="E7" s="42" t="inlineStr"/>
+      <c r="E7" s="49" t="inlineStr"/>
       <c r="F7" s="32" t="inlineStr">
         <is>
           <t>Term premium widens whether the Fed hikes or loses credibility. Trade 2, already in the book.</t>
@@ -33971,27 +35315,27 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="41" t="inlineStr">
+      <c r="A8" s="48" t="inlineStr">
         <is>
           <t>2 · Energy / terms of trade</t>
         </is>
       </c>
-      <c r="B8" s="42" t="inlineStr">
+      <c r="B8" s="49" t="inlineStr">
         <is>
           <t>Brent $72 → $102 → $88</t>
         </is>
       </c>
-      <c r="C8" s="42" t="inlineStr">
+      <c r="C8" s="49" t="inlineStr">
         <is>
           <t>JPY 2s10s bull steepener</t>
         </is>
       </c>
-      <c r="D8" s="42" t="inlineStr">
+      <c r="D8" s="49" t="inlineStr">
         <is>
           <t>Bull steepener</t>
         </is>
       </c>
-      <c r="E8" s="42" t="inlineStr"/>
+      <c r="E8" s="49" t="inlineStr"/>
       <c r="F8" s="32" t="inlineStr">
         <is>
           <t>Japan is the G7's largest net energy importer. The BoJ's own Outlook writes the terms-of-trade hit into its forecasts. This trade.</t>
@@ -33999,27 +35343,27 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="41" t="inlineStr">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>3 · Tariffs</t>
         </is>
       </c>
-      <c r="B9" s="42" t="inlineStr">
+      <c r="B9" s="49" t="inlineStr">
         <is>
           <t>10–12.5%, statutory</t>
         </is>
       </c>
-      <c r="C9" s="42" t="inlineStr">
+      <c r="C9" s="49" t="inlineStr">
         <is>
           <t>Japan vs Korea equity spread</t>
         </is>
       </c>
-      <c r="D9" s="42" t="inlineStr">
+      <c r="D9" s="49" t="inlineStr">
         <is>
           <t>Relative value</t>
         </is>
       </c>
-      <c r="E9" s="42" t="inlineStr"/>
+      <c r="E9" s="49" t="inlineStr"/>
       <c r="F9" s="32" t="inlineStr">
         <is>
           <t>A permanent margin tax, concentrated in Korean and Taiwanese electronics and near zero for Japanese domestic demand. Trade 1.</t>
@@ -34027,27 +35371,27 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="41" t="inlineStr">
+      <c r="A10" s="48" t="inlineStr">
         <is>
           <t>4 · Capital cycle</t>
         </is>
       </c>
-      <c r="B10" s="42" t="inlineStr">
+      <c r="B10" s="49" t="inlineStr">
         <is>
           <t>China DUV, ~$270bn</t>
         </is>
       </c>
-      <c r="C10" s="42" t="inlineStr">
+      <c r="C10" s="49" t="inlineStr">
         <is>
           <t>Short Korea semis</t>
         </is>
       </c>
-      <c r="D10" s="42" t="inlineStr">
+      <c r="D10" s="49" t="inlineStr">
         <is>
           <t>Directional</t>
         </is>
       </c>
-      <c r="E10" s="42" t="inlineStr"/>
+      <c r="E10" s="49" t="inlineStr"/>
       <c r="F10" s="32" t="inlineStr">
         <is>
           <t>A terminal-value event, not an earnings event. Trade 1's short leg.</t>
@@ -34101,27 +35445,27 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="41" t="inlineStr">
+      <c r="A16" s="48" t="inlineStr">
         <is>
           <t>JPY 2s10s bull steepener</t>
         </is>
       </c>
-      <c r="B16" s="42" t="inlineStr">
+      <c r="B16" s="49" t="inlineStr">
         <is>
           <t>Carry</t>
         </is>
       </c>
-      <c r="C16" s="42" t="inlineStr">
+      <c r="C16" s="49" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
       </c>
-      <c r="D16" s="42" t="inlineStr">
+      <c r="D16" s="49" t="inlineStr">
         <is>
           <t>Loses</t>
         </is>
       </c>
-      <c r="E16" s="42" t="inlineStr">
+      <c r="E16" s="49" t="inlineStr">
         <is>
           <t>Loses</t>
         </is>
@@ -34133,27 +35477,27 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="41" t="inlineStr">
+      <c r="A17" s="48" t="inlineStr">
         <is>
           <t>Trade 1 · long Japan banks</t>
         </is>
       </c>
-      <c r="B17" s="42" t="inlineStr">
+      <c r="B17" s="49" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
       </c>
-      <c r="C17" s="42" t="inlineStr">
+      <c r="C17" s="49" t="inlineStr">
         <is>
           <t>Loses</t>
         </is>
       </c>
-      <c r="D17" s="42" t="inlineStr">
+      <c r="D17" s="49" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
       </c>
-      <c r="E17" s="42" t="inlineStr">
+      <c r="E17" s="49" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
@@ -34165,27 +35509,27 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="41" t="inlineStr">
+      <c r="A18" s="48" t="inlineStr">
         <is>
           <t>Trade 2 · US 5s30s</t>
         </is>
       </c>
-      <c r="B18" s="42" t="inlineStr">
+      <c r="B18" s="49" t="inlineStr">
         <is>
           <t>Carry</t>
         </is>
       </c>
-      <c r="C18" s="42" t="inlineStr">
+      <c r="C18" s="49" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
       </c>
-      <c r="D18" s="42" t="inlineStr">
+      <c r="D18" s="49" t="inlineStr">
         <is>
           <t>Loses</t>
         </is>
       </c>
-      <c r="E18" s="42" t="inlineStr">
+      <c r="E18" s="49" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
@@ -34197,27 +35541,27 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="41" t="inlineStr">
+      <c r="A19" s="48" t="inlineStr">
         <is>
           <t>Trade 3 · gold call spread</t>
         </is>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B19" s="49" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="C19" s="42" t="inlineStr">
+      <c r="C19" s="49" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
       </c>
-      <c r="D19" s="42" t="inlineStr">
+      <c r="D19" s="49" t="inlineStr">
         <is>
           <t>Loses</t>
         </is>
       </c>
-      <c r="E19" s="42" t="inlineStr">
+      <c r="E19" s="49" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
@@ -34267,23 +35611,23 @@
       </c>
     </row>
     <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="41" t="inlineStr">
+      <c r="A26" s="48" t="inlineStr">
         <is>
           <t>JGB 10s30s</t>
         </is>
       </c>
-      <c r="B26" s="42" t="inlineStr">
+      <c r="B26" s="49" t="inlineStr">
         <is>
           <t>Flatteners — consensus</t>
         </is>
       </c>
-      <c r="C26" s="42" t="inlineStr">
+      <c r="C26" s="49" t="inlineStr">
         <is>
           <t>Not in it</t>
         </is>
       </c>
-      <c r="D26" s="42" t="inlineStr"/>
-      <c r="E26" s="42" t="inlineStr"/>
+      <c r="D26" s="49" t="inlineStr"/>
+      <c r="E26" s="49" t="inlineStr"/>
       <c r="F26" s="32" t="inlineStr">
         <is>
           <t>The long-end premium is technical, and the MoF is fixing the technical by cutting super-long issuance to a 17-year low. The street is right, and it is not our trade.</t>
@@ -34291,23 +35635,23 @@
       </c>
     </row>
     <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="41" t="inlineStr">
+      <c r="A27" s="48" t="inlineStr">
         <is>
           <t>JGB 2s10s</t>
         </is>
       </c>
-      <c r="B27" s="42" t="inlineStr">
+      <c r="B27" s="49" t="inlineStr">
         <is>
           <t>No consensus position</t>
         </is>
       </c>
-      <c r="C27" s="42" t="inlineStr">
+      <c r="C27" s="49" t="inlineStr">
         <is>
           <t>Bull steepener</t>
         </is>
       </c>
-      <c r="D27" s="42" t="inlineStr"/>
-      <c r="E27" s="42" t="inlineStr"/>
+      <c r="D27" s="49" t="inlineStr"/>
+      <c r="E27" s="49" t="inlineStr"/>
       <c r="F27" s="32" t="inlineStr">
         <is>
           <t>The front end is the fundamental curve — it is where the BoJ path lives. Nobody is positioned here. This is the opposite of the crowding problem on Trade 1.</t>
@@ -34315,23 +35659,23 @@
       </c>
     </row>
     <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="41" t="inlineStr">
+      <c r="A28" s="48" t="inlineStr">
         <is>
           <t>US / UK curves</t>
         </is>
       </c>
-      <c r="B28" s="42" t="inlineStr">
+      <c r="B28" s="49" t="inlineStr">
         <is>
           <t>Steepeners — consensus</t>
         </is>
       </c>
-      <c r="C28" s="42" t="inlineStr">
+      <c r="C28" s="49" t="inlineStr">
         <is>
           <t>Steepener (Trade 2)</t>
         </is>
       </c>
-      <c r="D28" s="42" t="inlineStr"/>
-      <c r="E28" s="42" t="inlineStr"/>
+      <c r="D28" s="49" t="inlineStr"/>
+      <c r="E28" s="49" t="inlineStr"/>
       <c r="F28" s="32" t="inlineStr">
         <is>
           <t>We are with the street here, and we should say so rather than pretend it is differentiated.</t>
@@ -34339,23 +35683,23 @@
       </c>
     </row>
     <row r="29" ht="34" customHeight="1">
-      <c r="A29" s="41" t="inlineStr">
+      <c r="A29" s="48" t="inlineStr">
         <is>
           <t>Japan banks</t>
         </is>
       </c>
-      <c r="B29" s="42" t="inlineStr">
+      <c r="B29" s="49" t="inlineStr">
         <is>
           <t>Long — crowded</t>
         </is>
       </c>
-      <c r="C29" s="42" t="inlineStr">
+      <c r="C29" s="49" t="inlineStr">
         <is>
           <t>Long (Trade 1)</t>
         </is>
       </c>
-      <c r="D29" s="42" t="inlineStr"/>
-      <c r="E29" s="42" t="inlineStr"/>
+      <c r="D29" s="49" t="inlineStr"/>
+      <c r="E29" s="49" t="inlineStr"/>
       <c r="F29" s="32" t="inlineStr">
         <is>
           <t>MUFG and SMFG NIMs expanding for the first time in a generation. Crowded, and volunteered as such in the macro deck.</t>
@@ -34650,7 +35994,7 @@
         <f>IFERROR((BDP($B58,"PX_LAST")-BDP($C58,"PX_LAST"))*100,"")</f>
         <v/>
       </c>
-      <c r="E58" s="43">
+      <c r="E58" s="50">
         <f>IFERROR(CurveSlope!H21,"")</f>
         <v/>
       </c>
@@ -34680,7 +36024,7 @@
         <f>IFERROR((BDP($B59,"PX_LAST")-BDP($C59,"PX_LAST"))*100,"")</f>
         <v/>
       </c>
-      <c r="E59" s="43">
+      <c r="E59" s="50">
         <f>IFERROR(CurveSlope!H18,"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add the Catalysts tab, and fix the Payoff tab's silent failure
Catalysts carries the dated Japan calendar to year-end with the 2-year move
each event produces against us and for us, and what the calendar adds up to.
The useful output is the last line: threat-to-confirm runs at about 1.45 to
one, and roughly 60% of the threat sits in the two meetings rather than in
the prints. The calendar is asymmetric against the position, which is worth
saying before being asked.

Payoff was computing off (outcome less entry), and the entry cell reads a
live Bloomberg chain. Off-terminal it came back empty and the tab produced
plausible numbers rather than errors. The payoff never needed the level —
it is a function of the two moves — so it now computes from those and
reconciles to hand calculation.
</commit_message>
<xml_diff>
--- a/JPY_Bull_Steepener.xlsx
+++ b/JPY_Bull_Steepener.xlsx
@@ -16,7 +16,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BullSteepener" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JPYEvidence" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payoff" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MacroLink" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalysts" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MacroLink" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="AsOf">Control!$B$6</definedName>
@@ -35,7 +36,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="dd-mmm-yyyy"/>
     <numFmt numFmtId="165" formatCode="+0.00;-0.00"/>
     <numFmt numFmtId="166" formatCode="+#,##0;-#,##0"/>
@@ -45,8 +46,10 @@
     <numFmt numFmtId="170" formatCode="dd-mmm-yy"/>
     <numFmt numFmtId="171" formatCode="0.0"/>
     <numFmt numFmtId="172" formatCode="+#,##0.0;-#,##0.0"/>
+    <numFmt numFmtId="173" formatCode="+#,##0.00;-#,##0.00"/>
+    <numFmt numFmtId="174" formatCode="+0%;-0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -102,6 +105,24 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00DB0011"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0000847F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00767576"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00DB0011"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -140,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -162,7 +183,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -205,11 +226,34 @@
     <xf numFmtId="9" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="172" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -1210,6 +1254,188 @@
                 </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:rPr>
+              <a:t>Expected value, bp, against net premium paid</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="DB0011"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Payoff'!$A$49:$A$55</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Payoff'!$B$49:$B$55</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <numFmt formatCode="+#,##0.0;-#,##0.0"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="1000" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Arial"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t/>
+              </a:r>
+              <a:endParaRPr sz="1000" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:endParaRPr>
+            </a:p>
+          </txPr>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="60"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D0CECE"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="950" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="767576"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="767576"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D0CECE"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="950" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="767576"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="767576"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+  <spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:noFill/>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:rPr>
               <a:t>Payoff by state, bp of 2s10s</a:t>
             </a:r>
           </a:p>
@@ -1424,7 +1650,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -1606,7 +1832,426 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>What each catalyst is worth to the 2-year, bp</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>2y move if it goes against us, bp</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="DB0011"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Catalysts'!$B$6:$B$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Catalysts'!$D$6:$D$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>2y move if it goes for us, bp</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="00847F"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Catalysts'!$B$6:$B$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Catalysts'!$E$6:$E$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <numFmt formatCode="+#,##0;-#,##0"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="1000" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Arial"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t/>
+              </a:r>
+              <a:endParaRPr sz="1000" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:endParaRPr>
+            </a:p>
+          </txPr>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="60"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D0CECE"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="950" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="767576"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="767576"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D0CECE"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="950" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="767576"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="767576"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+      <overlay val="0"/>
+      <txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:t/>
+          </a:r>
+          <a:endParaRPr sz="950" b="0">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:latin typeface="Arial"/>
+          </a:endParaRPr>
+        </a:p>
+      </txPr>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+  <spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:noFill/>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart17.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>Total range each catalyst can produce, bp</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="44546A"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Catalysts'!$B$6:$B$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Catalysts'!$F$6:$F$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <numFmt formatCode="#,##0"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="1000" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Arial"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t/>
+              </a:r>
+              <a:endParaRPr sz="1000" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:endParaRPr>
+            </a:p>
+          </txPr>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="60"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D0CECE"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="950" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="767576"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="767576"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D0CECE"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="950" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="767576"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="767576"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+  <spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:noFill/>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart18.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -1788,7 +2433,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart19.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -1970,7 +2615,189 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>Shunto settlement, % — annual</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="44546A"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'BOJPath'!$A$16:$A$21</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'BOJPath'!$E$16:$E$21</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <numFmt formatCode="0.00"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="1000" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Arial"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t/>
+              </a:r>
+              <a:endParaRPr sz="1000" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:endParaRPr>
+            </a:p>
+          </txPr>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="60"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D0CECE"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="950" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="767576"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="767576"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D0CECE"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="950" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="767576"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="950" b="0">
+              <a:solidFill>
+                <a:srgbClr val="767576"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+  <spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:noFill/>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart20.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -2195,188 +3022,6 @@
         </a:p>
       </txPr>
     </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-  <spPr>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-      <a:noFill/>
-      <a:prstDash val="solid"/>
-    </a:ln>
-  </spPr>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr sz="1200" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Arial"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr sz="1200" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Arial"/>
-              </a:rPr>
-              <a:t>Shunto settlement, % — annual</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="44546A"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'BOJPath'!$A$16:$A$21</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'BOJPath'!$E$16:$E$21</f>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <numFmt formatCode="0.00"/>
-          <txPr>
-            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:pPr>
-                <a:defRPr sz="1000" b="1">
-                  <a:solidFill>
-                    <a:srgbClr val="000000"/>
-                  </a:solidFill>
-                  <a:latin typeface="Arial"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:r>
-                <a:t/>
-              </a:r>
-              <a:endParaRPr sz="1000" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Arial"/>
-              </a:endParaRPr>
-            </a:p>
-          </txPr>
-          <showVal val="1"/>
-        </dLbls>
-        <gapWidth val="60"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
-            <a:solidFill>
-              <a:srgbClr val="D0CECE"/>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr sz="950" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="767576"/>
-                </a:solidFill>
-                <a:latin typeface="Arial"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="950" b="0">
-              <a:solidFill>
-                <a:srgbClr val="767576"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-            </a:endParaRPr>
-          </a:p>
-        </txPr>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
-            <a:solidFill>
-              <a:srgbClr val="D0CECE"/>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr sz="950" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="767576"/>
-                </a:solidFill>
-                <a:latin typeface="Arial"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="950" b="0">
-              <a:solidFill>
-                <a:srgbClr val="767576"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-            </a:endParaRPr>
-          </a:p>
-        </txPr>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -4726,7 +5371,7 @@
     <from>
       <col>9</col>
       <colOff>0</colOff>
-      <row>4</row>
+      <row>42</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3240000"/>
@@ -4748,7 +5393,7 @@
     <from>
       <col>9</col>
       <colOff>0</colOff>
-      <row>23</row>
+      <row>4</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3240000"/>
@@ -4766,10 +5411,81 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
 <file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7560000" cy="3960000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7560000" cy="3960000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -5129,7 +5845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5240,71 +5956,83 @@
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Payoff</t>
+          <t>Catalysts</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>What it makes by state of the world, an expected value for both expressions, sizing against the rates sleeve, and a falsification calendar with a date and a number on every line. Two charts.</t>
+          <t>The dated Japan calendar to year-end, with the 2-year move each event would produce against us and for us, and what the calendar adds up to. Two charts.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
+          <t>Payoff</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>What it makes by state of the world, an expected value for both expressions, sizing against the rates sleeve, and a falsification calendar with a date and a number on every line. Two charts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
           <t>MacroLink</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>The artefacts that tie the trade to the macro framing: channel-to-instrument map, scenario strip, positioning table, and three charts. Three charts, three tables.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>How to run it</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>1.  Open on the Bloomberg laptop and confirm the ribbon is present.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>2.  Control tab — set the as-of date, or leave =TODAY() for a live book.</t>
+          <t>1.  Open on the Bloomberg laptop and confirm the ribbon is present.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>3.  Bloomberg &gt; Refresh &gt; Refresh Entire Workbook.</t>
+          <t>2.  Control tab — set the as-of date, or leave =TODAY() for a live book.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>4.  Check the date alignment cell near the top of each tab reads 0 / OK before trusting a number.</t>
+          <t>3.  Bloomberg &gt; Refresh &gt; Refresh Entire Workbook.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="7" t="inlineStr">
         <is>
+          <t>4.  Check the date alignment cell near the top of each tab reads 0 / OK before trusting a number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="7" t="inlineStr">
+        <is>
           <t>5.  The charts redraw themselves — they point at the ranges the formulas spill into, not at pasted values.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>This file is a build artefact. It is generated by data-puller/build_data_puller.py alongside the full Q2 book and shares every sheet builder with it, so the two cannot disagree. Never repair it by hand — fix the script and rebuild, or the fix is lost the next time anyone regenerates it.</t>
         </is>
@@ -5316,6 +6044,489 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Japan risk catalysts, and what each one is worth</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled dates to year-end, with the 2-year move each would produce. The trade lives or dies on five of these.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="4" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>What it tests</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>2y if against us, bp</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>2y if for us, bp</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Range, bp</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>12 Aug 2026</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>Q2 GDP, preliminary</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>Whether growth is rolling</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" s="29" t="n">
+        <v>-4</v>
+      </c>
+      <c r="F6" s="29">
+        <f>IFERROR(D6-E6,"")</f>
+        <v/>
+      </c>
+      <c r="G6" s="61" t="inlineStr">
+        <is>
+          <t>Threat</t>
+        </is>
+      </c>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>Already out and against us — revised up to 0.8% annualised.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>18 Sep 2026</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>BoJ policy meeting</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>The path, not just the level</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="n">
+        <v>18</v>
+      </c>
+      <c r="E7" s="29" t="n">
+        <v>-22</v>
+      </c>
+      <c r="F7" s="29">
+        <f>IFERROR(D7-E7,"")</f>
+        <v/>
+      </c>
+      <c r="G7" s="61" t="inlineStr">
+        <is>
+          <t>Threat</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>A hike WITH hawkish guidance is the bad outcome. A hike framed as one-and-done is the entry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>19 Sep 2026</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>August national CPI</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>Core-core, the thesis measure</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="29" t="n">
+        <v>-14</v>
+      </c>
+      <c r="F8" s="29">
+        <f>IFERROR(D8-E8,"")</f>
+        <v/>
+      </c>
+      <c r="G8" s="62" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>First of three. Below 1.8% and the hiking case weakens materially.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>20 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>September national CPI</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>Core-core, second print</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" s="29" t="n">
+        <v>-14</v>
+      </c>
+      <c r="F9" s="29">
+        <f>IFERROR(D9-E9,"")</f>
+        <v/>
+      </c>
+      <c r="G9" s="62" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Two prints make a direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>BoJ meeting and Outlook Report</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>The FY27 CPI forecast</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="E10" s="29" t="n">
+        <v>-28</v>
+      </c>
+      <c r="F10" s="29">
+        <f>IFERROR(D10-E10,"")</f>
+        <v/>
+      </c>
+      <c r="G10" s="61" t="inlineStr">
+        <is>
+          <t>Threat</t>
+        </is>
+      </c>
+      <c r="H10" s="16" t="inlineStr">
+        <is>
+          <t>The single largest event on this calendar. An upward FY27 revision ends the trade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>20 Nov 2026</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>October national CPI</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>Core-core, third print</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" s="29" t="n">
+        <v>-16</v>
+      </c>
+      <c r="F11" s="29">
+        <f>IFERROR(D11-E11,"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="62" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>By here the direction is established either way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>MoF FY27 issuance plan</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>Super-long supply</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="29" t="n">
+        <v>-2</v>
+      </c>
+      <c r="F12" s="29">
+        <f>IFERROR(D12-E12,"")</f>
+        <v/>
+      </c>
+      <c r="G12" s="63" t="inlineStr">
+        <is>
+          <t>Context</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>Moves the 30y, barely touches the 2y. It is why we are in 2s10s and not 2s30s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>18 Dec 2026</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>BoJ policy meeting</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>The last of the year</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="n">
+        <v>16</v>
+      </c>
+      <c r="E13" s="29" t="n">
+        <v>-20</v>
+      </c>
+      <c r="F13" s="29">
+        <f>IFERROR(D13-E13,"")</f>
+        <v/>
+      </c>
+      <c r="G13" s="61" t="inlineStr">
+        <is>
+          <t>Threat</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Only live if September and October passed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>What the calendar adds up to</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>Worst case, all threats against us, bp</t>
+        </is>
+      </c>
+      <c r="D17" s="29">
+        <f>IFERROR(SUMIF($G$6:$G$13,"Threat",$D$6:$D$13),"")</f>
+        <v/>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Every meeting hawkish. This is the tail, not the base case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>Best case, all confirms for us, bp</t>
+        </is>
+      </c>
+      <c r="D18" s="29">
+        <f>IFERROR(SUMIF($G$6:$G$13,"Confirm",$E$6:$E$13),"")</f>
+        <v/>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>Three core-core prints all soft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>Largest single threat, bp</t>
+        </is>
+      </c>
+      <c r="D19" s="29">
+        <f>IFERROR(MAX($D$6:$D$13),"")</f>
+        <v/>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>The 29 October Outlook Report, and it is not close.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>Meetings as a share of total threat</t>
+        </is>
+      </c>
+      <c r="D20" s="31">
+        <f>IFERROR(SUMIF($B$6:$B$13,"BoJ*",$D$6:$D$13)/SUM($D$6:$D$13),"")</f>
+        <v/>
+      </c>
+      <c r="H20" s="16" t="inlineStr">
+        <is>
+          <t>The risk is concentrated in the meetings rather than the prints, which is why the entry trigger is a meeting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>Threat-to-confirm ratio</t>
+        </is>
+      </c>
+      <c r="D21" s="23">
+        <f>IFERROR(SUMIF($G$6:$G$13,"Threat",$D$6:$D$13)/ABS(SUMIF($G$6:$G$13,"Confirm",$E$6:$E$13)),"")</f>
+        <v/>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>Above 1 means the calendar is asymmetric against us — worth saying out loud rather than being asked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>The 2-year moves are estimates, sized off what the front end holds: about 55bp of priced hikes, so a full repricing is that order and a single delivered hike is roughly a quarter of it. They are here to rank the calendar, not to price a position — the ranking is robust to being wrong about any one of them.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5393,27 +6604,27 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="51" t="inlineStr">
+      <c r="A7" s="64" t="inlineStr">
         <is>
           <t>1 · Fed / discount rate</t>
         </is>
       </c>
-      <c r="B7" s="52" t="inlineStr">
+      <c r="B7" s="65" t="inlineStr">
         <is>
           <t>UST 10y 3.97 → 4.71%</t>
         </is>
       </c>
-      <c r="C7" s="52" t="inlineStr">
+      <c r="C7" s="65" t="inlineStr">
         <is>
           <t>US 5s30s steepener</t>
         </is>
       </c>
-      <c r="D7" s="52" t="inlineStr">
+      <c r="D7" s="65" t="inlineStr">
         <is>
           <t>Bear steepener</t>
         </is>
       </c>
-      <c r="E7" s="52" t="inlineStr"/>
+      <c r="E7" s="65" t="inlineStr"/>
       <c r="F7" s="16" t="inlineStr">
         <is>
           <t>Term premium widens whether the Fed hikes or loses credibility. Trade 2, already in the book.</t>
@@ -5421,27 +6632,27 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="51" t="inlineStr">
+      <c r="A8" s="64" t="inlineStr">
         <is>
           <t>2 · Energy / terms of trade</t>
         </is>
       </c>
-      <c r="B8" s="52" t="inlineStr">
+      <c r="B8" s="65" t="inlineStr">
         <is>
           <t>Brent $72 → $102 → $88</t>
         </is>
       </c>
-      <c r="C8" s="52" t="inlineStr">
+      <c r="C8" s="65" t="inlineStr">
         <is>
           <t>JPY 2s10s bull steepener</t>
         </is>
       </c>
-      <c r="D8" s="52" t="inlineStr">
+      <c r="D8" s="65" t="inlineStr">
         <is>
           <t>Bull steepener</t>
         </is>
       </c>
-      <c r="E8" s="52" t="inlineStr"/>
+      <c r="E8" s="65" t="inlineStr"/>
       <c r="F8" s="16" t="inlineStr">
         <is>
           <t>Japan is the G7's largest net energy importer. The BoJ's own Outlook writes the terms-of-trade hit into its forecasts. This trade.</t>
@@ -5449,27 +6660,27 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="51" t="inlineStr">
+      <c r="A9" s="64" t="inlineStr">
         <is>
           <t>3 · Tariffs</t>
         </is>
       </c>
-      <c r="B9" s="52" t="inlineStr">
+      <c r="B9" s="65" t="inlineStr">
         <is>
           <t>10–12.5%, statutory</t>
         </is>
       </c>
-      <c r="C9" s="52" t="inlineStr">
+      <c r="C9" s="65" t="inlineStr">
         <is>
           <t>Japan vs Korea equity spread</t>
         </is>
       </c>
-      <c r="D9" s="52" t="inlineStr">
+      <c r="D9" s="65" t="inlineStr">
         <is>
           <t>Relative value</t>
         </is>
       </c>
-      <c r="E9" s="52" t="inlineStr"/>
+      <c r="E9" s="65" t="inlineStr"/>
       <c r="F9" s="16" t="inlineStr">
         <is>
           <t>A permanent margin tax, concentrated in Korean and Taiwanese electronics and near zero for Japanese domestic demand. Trade 1.</t>
@@ -5477,27 +6688,27 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="51" t="inlineStr">
+      <c r="A10" s="64" t="inlineStr">
         <is>
           <t>4 · Capital cycle</t>
         </is>
       </c>
-      <c r="B10" s="52" t="inlineStr">
+      <c r="B10" s="65" t="inlineStr">
         <is>
           <t>China DUV, ~$270bn</t>
         </is>
       </c>
-      <c r="C10" s="52" t="inlineStr">
+      <c r="C10" s="65" t="inlineStr">
         <is>
           <t>Short Korea semis</t>
         </is>
       </c>
-      <c r="D10" s="52" t="inlineStr">
+      <c r="D10" s="65" t="inlineStr">
         <is>
           <t>Directional</t>
         </is>
       </c>
-      <c r="E10" s="52" t="inlineStr"/>
+      <c r="E10" s="65" t="inlineStr"/>
       <c r="F10" s="16" t="inlineStr">
         <is>
           <t>A terminal-value event, not an earnings event. Trade 1's short leg.</t>
@@ -5551,27 +6762,27 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="51" t="inlineStr">
+      <c r="A16" s="64" t="inlineStr">
         <is>
           <t>JPY 2s10s bull steepener</t>
         </is>
       </c>
-      <c r="B16" s="52" t="inlineStr">
+      <c r="B16" s="65" t="inlineStr">
         <is>
           <t>Carry</t>
         </is>
       </c>
-      <c r="C16" s="52" t="inlineStr">
+      <c r="C16" s="65" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
       </c>
-      <c r="D16" s="52" t="inlineStr">
+      <c r="D16" s="65" t="inlineStr">
         <is>
           <t>Loses</t>
         </is>
       </c>
-      <c r="E16" s="52" t="inlineStr">
+      <c r="E16" s="65" t="inlineStr">
         <is>
           <t>Loses</t>
         </is>
@@ -5583,27 +6794,27 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="51" t="inlineStr">
+      <c r="A17" s="64" t="inlineStr">
         <is>
           <t>Trade 1 · long Japan banks</t>
         </is>
       </c>
-      <c r="B17" s="52" t="inlineStr">
+      <c r="B17" s="65" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
       </c>
-      <c r="C17" s="52" t="inlineStr">
+      <c r="C17" s="65" t="inlineStr">
         <is>
           <t>Loses</t>
         </is>
       </c>
-      <c r="D17" s="52" t="inlineStr">
+      <c r="D17" s="65" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
       </c>
-      <c r="E17" s="52" t="inlineStr">
+      <c r="E17" s="65" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
@@ -5615,27 +6826,27 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="51" t="inlineStr">
+      <c r="A18" s="64" t="inlineStr">
         <is>
           <t>Trade 2 · US 5s30s</t>
         </is>
       </c>
-      <c r="B18" s="52" t="inlineStr">
+      <c r="B18" s="65" t="inlineStr">
         <is>
           <t>Carry</t>
         </is>
       </c>
-      <c r="C18" s="52" t="inlineStr">
+      <c r="C18" s="65" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
       </c>
-      <c r="D18" s="52" t="inlineStr">
+      <c r="D18" s="65" t="inlineStr">
         <is>
           <t>Loses</t>
         </is>
       </c>
-      <c r="E18" s="52" t="inlineStr">
+      <c r="E18" s="65" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
@@ -5647,27 +6858,27 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="51" t="inlineStr">
+      <c r="A19" s="64" t="inlineStr">
         <is>
           <t>Trade 3 · gold call spread</t>
         </is>
       </c>
-      <c r="B19" s="52" t="inlineStr">
+      <c r="B19" s="65" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="C19" s="52" t="inlineStr">
+      <c r="C19" s="65" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
       </c>
-      <c r="D19" s="52" t="inlineStr">
+      <c r="D19" s="65" t="inlineStr">
         <is>
           <t>Loses</t>
         </is>
       </c>
-      <c r="E19" s="52" t="inlineStr">
+      <c r="E19" s="65" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
@@ -5717,23 +6928,23 @@
       </c>
     </row>
     <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="51" t="inlineStr">
+      <c r="A26" s="64" t="inlineStr">
         <is>
           <t>JGB 10s30s</t>
         </is>
       </c>
-      <c r="B26" s="52" t="inlineStr">
+      <c r="B26" s="65" t="inlineStr">
         <is>
           <t>Flatteners — consensus</t>
         </is>
       </c>
-      <c r="C26" s="52" t="inlineStr">
+      <c r="C26" s="65" t="inlineStr">
         <is>
           <t>Not in it</t>
         </is>
       </c>
-      <c r="D26" s="52" t="inlineStr"/>
-      <c r="E26" s="52" t="inlineStr"/>
+      <c r="D26" s="65" t="inlineStr"/>
+      <c r="E26" s="65" t="inlineStr"/>
       <c r="F26" s="16" t="inlineStr">
         <is>
           <t>The long-end premium is technical, and the MoF is fixing the technical by cutting super-long issuance to a 17-year low. The street is right, and it is not our trade.</t>
@@ -5741,23 +6952,23 @@
       </c>
     </row>
     <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="51" t="inlineStr">
+      <c r="A27" s="64" t="inlineStr">
         <is>
           <t>JGB 2s10s</t>
         </is>
       </c>
-      <c r="B27" s="52" t="inlineStr">
+      <c r="B27" s="65" t="inlineStr">
         <is>
           <t>No consensus position</t>
         </is>
       </c>
-      <c r="C27" s="52" t="inlineStr">
+      <c r="C27" s="65" t="inlineStr">
         <is>
           <t>Bull steepener</t>
         </is>
       </c>
-      <c r="D27" s="52" t="inlineStr"/>
-      <c r="E27" s="52" t="inlineStr"/>
+      <c r="D27" s="65" t="inlineStr"/>
+      <c r="E27" s="65" t="inlineStr"/>
       <c r="F27" s="16" t="inlineStr">
         <is>
           <t>The front end is the fundamental curve — it is where the BoJ path lives. Nobody is positioned here. This is the opposite of the crowding problem on Trade 1.</t>
@@ -5765,23 +6976,23 @@
       </c>
     </row>
     <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="51" t="inlineStr">
+      <c r="A28" s="64" t="inlineStr">
         <is>
           <t>US / UK curves</t>
         </is>
       </c>
-      <c r="B28" s="52" t="inlineStr">
+      <c r="B28" s="65" t="inlineStr">
         <is>
           <t>Steepeners — consensus</t>
         </is>
       </c>
-      <c r="C28" s="52" t="inlineStr">
+      <c r="C28" s="65" t="inlineStr">
         <is>
           <t>Steepener (Trade 2)</t>
         </is>
       </c>
-      <c r="D28" s="52" t="inlineStr"/>
-      <c r="E28" s="52" t="inlineStr"/>
+      <c r="D28" s="65" t="inlineStr"/>
+      <c r="E28" s="65" t="inlineStr"/>
       <c r="F28" s="16" t="inlineStr">
         <is>
           <t>We are with the street here, and we should say so rather than pretend it is differentiated.</t>
@@ -5789,23 +7000,23 @@
       </c>
     </row>
     <row r="29" ht="34" customHeight="1">
-      <c r="A29" s="51" t="inlineStr">
+      <c r="A29" s="64" t="inlineStr">
         <is>
           <t>Japan banks</t>
         </is>
       </c>
-      <c r="B29" s="52" t="inlineStr">
+      <c r="B29" s="65" t="inlineStr">
         <is>
           <t>Long — crowded</t>
         </is>
       </c>
-      <c r="C29" s="52" t="inlineStr">
+      <c r="C29" s="65" t="inlineStr">
         <is>
           <t>Long (Trade 1)</t>
         </is>
       </c>
-      <c r="D29" s="52" t="inlineStr"/>
-      <c r="E29" s="52" t="inlineStr"/>
+      <c r="D29" s="65" t="inlineStr"/>
+      <c r="E29" s="65" t="inlineStr"/>
       <c r="F29" s="16" t="inlineStr">
         <is>
           <t>MUFG and SMFG NIMs expanding for the first time in a generation. Crowded, and volunteered as such in the macro deck.</t>
@@ -6100,7 +7311,7 @@
         <f>IFERROR((BDP($B58,"PX_LAST")-BDP($C58,"PX_LAST"))*100,"")</f>
         <v/>
       </c>
-      <c r="E58" s="53">
+      <c r="E58" s="66">
         <f>IFERROR(CurveSlope!H21,"")</f>
         <v/>
       </c>
@@ -6130,7 +7341,7 @@
         <f>IFERROR((BDP($B59,"PX_LAST")-BDP($C59,"PX_LAST"))*100,"")</f>
         <v/>
       </c>
-      <c r="E59" s="53">
+      <c r="E59" s="66">
         <f>IFERROR(CurveSlope!H18,"")</f>
         <v/>
       </c>
@@ -35716,7 +36927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -35847,26 +37058,26 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="H11" s="16" t="inlineStr">
         <is>
-          <t>6m conditional bull steepener, receiver spread. JPY swaptions are quoted in NORMAL (Bachelier) vol in basis points, so price it off the vol surface and put the premium here in bp of notional. 18 is a placeholder until you do.</t>
+          <t>NET premium of the receiver spread — the 6m2y bought less the 6m10y sold. JPY swaptions quote in NORMAL (Bachelier) vol in basis points, so price both legs off the surface and put the net here. Compare it with the breakeven below before doing anything else.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Conditional strike, bp of steepening</t>
+          <t>Conditional strike offset, bp</t>
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H12" s="16" t="inlineStr">
         <is>
-          <t>How far the curve must steepen before the structure pays.</t>
+          <t>Zero because the structure is struck AT THE MONEY FORWARD. Raise it only if you deliberately cheapen the structure by striking out — and note what that does to the breakeven.</t>
         </is>
       </c>
     </row>
@@ -35937,7 +37148,7 @@
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>2s10s outcome</t>
+          <t>2s10s level</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
@@ -35972,15 +37183,15 @@
         <v>-3</v>
       </c>
       <c r="E21" s="38">
-        <f>IFERROR($B$6+(D21-C21),"")</f>
+        <f>IF(ISNUMBER($B$6),$B$6+(D21-C21),"refresh for level")</f>
         <v/>
       </c>
       <c r="F21" s="29">
-        <f>IFERROR((E21-$B$6)+$B$9*$B$10,"")</f>
+        <f>IFERROR((D21-C21)+IF(ISNUMBER($B$9),$B$9,0)*$B$10,"")</f>
         <v/>
       </c>
       <c r="G21" s="29">
-        <f>IFERROR(IF(C21&lt;0,MAX(0,(E21-$B$6)-$B$12),0)-$B$11,"")</f>
+        <f>IFERROR(IF(C21&lt;0,MAX(0,(D21-C21)-$B$12),0)-$B$11,"")</f>
         <v/>
       </c>
       <c r="H21" s="16" t="inlineStr">
@@ -36005,15 +37216,15 @@
         <v>2</v>
       </c>
       <c r="E22" s="38">
-        <f>IFERROR($B$6+(D22-C22),"")</f>
+        <f>IF(ISNUMBER($B$6),$B$6+(D22-C22),"refresh for level")</f>
         <v/>
       </c>
       <c r="F22" s="29">
-        <f>IFERROR((E22-$B$6)+$B$9*$B$10,"")</f>
+        <f>IFERROR((D22-C22)+IF(ISNUMBER($B$9),$B$9,0)*$B$10,"")</f>
         <v/>
       </c>
       <c r="G22" s="29">
-        <f>IFERROR(IF(C22&lt;0,MAX(0,(E22-$B$6)-$B$12),0)-$B$11,"")</f>
+        <f>IFERROR(IF(C22&lt;0,MAX(0,(D22-C22)-$B$12),0)-$B$11,"")</f>
         <v/>
       </c>
       <c r="H22" s="16" t="inlineStr">
@@ -36038,15 +37249,15 @@
         <v>37</v>
       </c>
       <c r="E23" s="38">
-        <f>IFERROR($B$6+(D23-C23),"")</f>
+        <f>IF(ISNUMBER($B$6),$B$6+(D23-C23),"refresh for level")</f>
         <v/>
       </c>
       <c r="F23" s="29">
-        <f>IFERROR((E23-$B$6)+$B$9*$B$10,"")</f>
+        <f>IFERROR((D23-C23)+IF(ISNUMBER($B$9),$B$9,0)*$B$10,"")</f>
         <v/>
       </c>
       <c r="G23" s="29">
-        <f>IFERROR(IF(C23&lt;0,MAX(0,(E23-$B$6)-$B$12),0)-$B$11,"")</f>
+        <f>IFERROR(IF(C23&lt;0,MAX(0,(D23-C23)-$B$12),0)-$B$11,"")</f>
         <v/>
       </c>
       <c r="H23" s="16" t="inlineStr">
@@ -36071,15 +37282,15 @@
         <v>7</v>
       </c>
       <c r="E24" s="38">
-        <f>IFERROR($B$6+(D24-C24),"")</f>
+        <f>IF(ISNUMBER($B$6),$B$6+(D24-C24),"refresh for level")</f>
         <v/>
       </c>
       <c r="F24" s="29">
-        <f>IFERROR((E24-$B$6)+$B$9*$B$10,"")</f>
+        <f>IFERROR((D24-C24)+IF(ISNUMBER($B$9),$B$9,0)*$B$10,"")</f>
         <v/>
       </c>
       <c r="G24" s="29">
-        <f>IFERROR(IF(C24&lt;0,MAX(0,(E24-$B$6)-$B$12),0)-$B$11,"")</f>
+        <f>IFERROR(IF(C24&lt;0,MAX(0,(D24-C24)-$B$12),0)-$B$11,"")</f>
         <v/>
       </c>
       <c r="H24" s="16" t="inlineStr">
@@ -36104,15 +37315,15 @@
         <v>-28</v>
       </c>
       <c r="E25" s="38">
-        <f>IFERROR($B$6+(D25-C25),"")</f>
+        <f>IF(ISNUMBER($B$6),$B$6+(D25-C25),"refresh for level")</f>
         <v/>
       </c>
       <c r="F25" s="29">
-        <f>IFERROR((E25-$B$6)+$B$9*$B$10,"")</f>
+        <f>IFERROR((D25-C25)+IF(ISNUMBER($B$9),$B$9,0)*$B$10,"")</f>
         <v/>
       </c>
       <c r="G25" s="29">
-        <f>IFERROR(IF(C25&lt;0,MAX(0,(E25-$B$6)-$B$12),0)-$B$11,"")</f>
+        <f>IFERROR(IF(C25&lt;0,MAX(0,(D25-C25)-$B$12),0)-$B$11,"")</f>
         <v/>
       </c>
       <c r="H25" s="16" t="inlineStr">
@@ -36246,135 +37457,176 @@
         <v/>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>Sizing</t>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>The pricing condition — the number this trade turns on</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>The conditional only has intrinsic value where the 2-year rallies. Its expected value is therefore the probability-weighted intrinsic in those states, less the premium paid in every state. Setting that to zero gives the most you can pay and still have a trade. It is not a wide margin, and pretending otherwise is how a structure gets bought at a level that cannot work.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="22" t="inlineStr">
-        <is>
-          <t>Rates sleeve, $m</t>
-        </is>
-      </c>
-      <c r="B40" s="35">
-        <f>IFERROR($B$13*$B$14,"")</f>
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Probability-weighted intrinsic, bp</t>
+        </is>
+      </c>
+      <c r="B40" s="48">
+        <f>IFERROR(SUMPRODUCT($B$21:$B$25,$G$21:$G$25)+$B$11,"")</f>
         <v/>
       </c>
       <c r="H40" s="16" t="inlineStr">
         <is>
-          <t>The sleeve this trade shares with the US 5s30s.</t>
+          <t>What the structure is worth before paying for it.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="22" t="inlineStr">
-        <is>
-          <t>Distance to stop, bp</t>
-        </is>
-      </c>
-      <c r="B41" s="37">
-        <f>IFERROR($B$6-$B$8,"")</f>
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>Breakeven premium, bp</t>
+        </is>
+      </c>
+      <c r="B41" s="48">
+        <f>IFERROR($B$40,"")</f>
         <v/>
       </c>
       <c r="H41" s="16" t="inlineStr">
         <is>
-          <t>Entry less stop.</t>
+          <t>Pay more than this and the expected value is negative. Full stop.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="22" t="inlineStr">
-        <is>
-          <t>Cash — max loss at stop, $m</t>
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>Premium actually paid, bp</t>
         </is>
       </c>
       <c r="B42" s="48">
-        <f>IFERROR($B$40*ABS($B$41)/10000*10,"")</f>
+        <f>IFERROR($B$11,"")</f>
         <v/>
       </c>
       <c r="H42" s="16" t="inlineStr">
         <is>
-          <t>At a DV01 sized so a 10bp adverse move costs 0.1% of the sleeve. Replace the factor with your desk's DV01 convention.</t>
+          <t>From the input block above.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="22" t="inlineStr">
-        <is>
-          <t>Cash — max loss, % of book</t>
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>Headroom, bp</t>
         </is>
       </c>
       <c r="B43" s="49">
-        <f>IFERROR($B$42/$B$13,"")</f>
+        <f>IFERROR($B$40-$B$11,"")</f>
         <v/>
       </c>
       <c r="H43" s="16" t="inlineStr">
         <is>
-          <t>The number the PM actually asks for.</t>
+          <t>Negative means do not do the trade at this price.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="22" t="inlineStr">
-        <is>
-          <t>Conditional — max loss, $m</t>
-        </is>
-      </c>
-      <c r="B44" s="48">
-        <f>IFERROR($B$40*$B$11/10000*10,"")</f>
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>Expected return on premium</t>
+        </is>
+      </c>
+      <c r="B44" s="50">
+        <f>IFERROR(($B$40-$B$11)/$B$11,"")</f>
         <v/>
       </c>
       <c r="H44" s="16" t="inlineStr">
         <is>
-          <t>Premium only, and it is known on day one.</t>
+          <t>The number to quote. Expected value per unit of capital at risk over six months, which is the honest denominator for a defined-premium structure — not basis points of notional.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="22" t="inlineStr">
-        <is>
-          <t>Conditional — max loss, % of book</t>
-        </is>
-      </c>
-      <c r="B45" s="49">
-        <f>IFERROR($B$44/$B$13,"")</f>
-        <v/>
-      </c>
-      <c r="H45" s="16" t="inlineStr">
-        <is>
-          <t>Pre-sized, no stop required, survives a gap.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="B45" s="18" t="n"/>
+      <c r="H45" s="16">
+        <f>IF($B$43="","",IF($B$43&gt;0,"BUY — priced inside the breakeven","DO NOT BUY at this premium. Either strike it differently, wait for a cheaper vol, or drop the trade."))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Expected value against the premium paid</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="51" t="inlineStr">
         <is>
           <t>The falsification calendar — dated, with the number</t>
         </is>
       </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>Expected value, bp</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Return on premium</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="A49" s="16" t="inlineStr">
         <is>
           <t>The July minutes show several Board members expecting inflation to accelerate significantly in the second half of the fiscal year, and two favouring faster hikes on firms' willingness to raise prices. That is the strongest argument against this trade and it is testable on a known date. Our reading is that broad-based price increases are cost pass-through from the same crude shock the April Outlook says will wane — so core-core is the arbiter, not headline.</t>
         </is>
       </c>
+      <c r="B49" s="47">
+        <f>IFERROR($B$40-A49,"")</f>
+        <v/>
+      </c>
+      <c r="C49" s="52">
+        <f>IFERROR(($B$40-A49)/A49,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="B50" s="47">
+        <f>IFERROR($B$40-A50,"")</f>
+        <v/>
+      </c>
+      <c r="C50" s="52">
+        <f>IFERROR(($B$40-A50)/A50,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="9" t="inlineStr">
+      <c r="A51" s="53" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B51" s="9" t="inlineStr">
+      <c r="B51" s="54" t="inlineStr">
         <is>
           <t>Event</t>
         </is>
       </c>
-      <c r="C51" s="9" t="inlineStr">
+      <c r="C51" s="55" t="inlineStr">
         <is>
           <t>What kills the trade</t>
         </is>
@@ -36395,12 +37647,12 @@
           <t>18 Sep 2026</t>
         </is>
       </c>
-      <c r="B52" s="22" t="inlineStr">
+      <c r="B52" s="56" t="inlineStr">
         <is>
           <t>BoJ policy meeting</t>
         </is>
       </c>
-      <c r="C52" s="50" t="inlineStr">
+      <c r="C52" s="57" t="inlineStr">
         <is>
           <t>A hike delivered WITH hawkish guidance on the path</t>
         </is>
@@ -36421,12 +37673,12 @@
           <t>Sep / Oct / Nov</t>
         </is>
       </c>
-      <c r="B53" s="22" t="inlineStr">
+      <c r="B53" s="56" t="inlineStr">
         <is>
           <t>National core-core CPI, monthly</t>
         </is>
       </c>
-      <c r="C53" s="50" t="inlineStr">
+      <c r="C53" s="57" t="inlineStr">
         <is>
           <t>Two consecutive prints back above 2.2% and rising</t>
         </is>
@@ -36447,12 +37699,12 @@
           <t>29 Oct 2026</t>
         </is>
       </c>
-      <c r="B54" s="22" t="inlineStr">
+      <c r="B54" s="56" t="inlineStr">
         <is>
           <t>BoJ policy meeting and Outlook Report</t>
         </is>
       </c>
-      <c r="C54" s="50" t="inlineStr">
+      <c r="C54" s="57" t="inlineStr">
         <is>
           <t>The FY27 CPI forecast revised UP</t>
         </is>
@@ -36473,12 +37725,12 @@
           <t>Monthly</t>
         </is>
       </c>
-      <c r="B55" s="22" t="inlineStr">
+      <c r="B55" s="56" t="inlineStr">
         <is>
           <t>USD/JPY against 165</t>
         </is>
       </c>
-      <c r="C55" s="50" t="inlineStr">
+      <c r="C55" s="57" t="inlineStr">
         <is>
           <t>Through 165 and holding — the BoJ hikes for FX regardless of growth</t>
         </is>
@@ -36504,7 +37756,7 @@
           <t>Real wages and household spending</t>
         </is>
       </c>
-      <c r="C56" s="50" t="inlineStr">
+      <c r="C56" s="58" t="inlineStr">
         <is>
           <t>Spending turns positive while real wages keep rising</t>
         </is>
@@ -36530,7 +37782,7 @@
           <t>Shunto first tally</t>
         </is>
       </c>
-      <c r="C57" s="50" t="inlineStr">
+      <c r="C57" s="58" t="inlineStr">
         <is>
           <t>Above 5.5% again, making the wage impulse durable</t>
         </is>
@@ -36545,10 +37797,106 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Sizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="22" t="inlineStr">
+        <is>
+          <t>Rates sleeve, $m</t>
+        </is>
+      </c>
+      <c r="B59" s="35">
+        <f>IFERROR($B$13*$B$14,"")</f>
+        <v/>
+      </c>
+      <c r="H59" s="16" t="inlineStr">
+        <is>
+          <t>The sleeve this trade shares with the US 5s30s.</t>
+        </is>
+      </c>
+    </row>
     <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="A60" s="16" t="inlineStr">
         <is>
           <t>Every line has a date and a number. A thesis without either is a view, and a view is not a trade — it is the thing you defend after it has gone wrong.</t>
+        </is>
+      </c>
+      <c r="B60" s="37">
+        <f>IFERROR($B$6-$B$8,"")</f>
+        <v/>
+      </c>
+      <c r="H60" s="16" t="inlineStr">
+        <is>
+          <t>Entry less stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="22" t="inlineStr">
+        <is>
+          <t>Cash — max loss at stop, $m</t>
+        </is>
+      </c>
+      <c r="B61" s="59">
+        <f>IFERROR($B$59*ABS($B$60)/10000*10,"")</f>
+        <v/>
+      </c>
+      <c r="H61" s="16" t="inlineStr">
+        <is>
+          <t>At a DV01 sized so a 10bp adverse move costs 0.1% of the sleeve. Replace the factor with your desk's DV01 convention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="22" t="inlineStr">
+        <is>
+          <t>Cash — max loss, % of book</t>
+        </is>
+      </c>
+      <c r="B62" s="60">
+        <f>IFERROR($B$61/$B$13,"")</f>
+        <v/>
+      </c>
+      <c r="H62" s="16" t="inlineStr">
+        <is>
+          <t>The number the PM actually asks for.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="22" t="inlineStr">
+        <is>
+          <t>Conditional — max loss, $m</t>
+        </is>
+      </c>
+      <c r="B63" s="59">
+        <f>IFERROR($B$59*$B$11/10000*10,"")</f>
+        <v/>
+      </c>
+      <c r="H63" s="16" t="inlineStr">
+        <is>
+          <t>Premium only, and it is known on day one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="22" t="inlineStr">
+        <is>
+          <t>Conditional — max loss, % of book</t>
+        </is>
+      </c>
+      <c r="B64" s="60">
+        <f>IFERROR($B$63/$B$13,"")</f>
+        <v/>
+      </c>
+      <c r="H64" s="16" t="inlineStr">
+        <is>
+          <t>Pre-sized, no stop required, survives a gap.</t>
         </is>
       </c>
     </row>

</xml_diff>